<commit_message>
Pantheon der 8 hinzugefügt
</commit_message>
<xml_diff>
--- a/docs/Buch Bayrische Nächte/Zeitlinie.xlsx
+++ b/docs/Buch Bayrische Nächte/Zeitlinie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{074B868B-F1AC-409B-99A3-EFAF7C2913BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B437D2A-10C0-4FB1-AC11-5404F361E360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="90">
   <si>
     <t>Year</t>
   </si>
@@ -201,9 +201,6 @@
     <t>Aelxander goes to Munich to start studying at TUM at 16 years of age</t>
   </si>
   <si>
-    <t>Prologe</t>
-  </si>
-  <si>
     <t>Chaper 10</t>
   </si>
   <si>
@@ -233,16 +230,76 @@
     <t>Marina, Wilheml Freiherr, Philipp</t>
   </si>
   <si>
-    <t>Marina, Wilhelm, Philipp, Christoff, Gundel</t>
-  </si>
-  <si>
-    <t>Continuing Marina wakes up and remmebers the Coutns boat, searching in it for clues</t>
-  </si>
-  <si>
     <t>Marina, Gundel</t>
   </si>
   <si>
     <t>Josef, August, Ingenheim, Ashen-One, Lady of the Cult</t>
+  </si>
+  <si>
+    <t>Continuing Marina wakes up and remmebers the Counts boat, searching in it for clues</t>
+  </si>
+  <si>
+    <t>Friedrich, Marina, Alexander, Anna, Sabine, Helene Berthold, Nai, Sir Charles, etc.</t>
+  </si>
+  <si>
+    <t>Chapter 17</t>
+  </si>
+  <si>
+    <t>Chapter 14</t>
+  </si>
+  <si>
+    <t>Friedrich is talking with his demented mom about life</t>
+  </si>
+  <si>
+    <t>Friedrich, Walburga Pfeiffer</t>
+  </si>
+  <si>
+    <t>Marina, Wilhelm, Philipp, Christoff Bauer, Gundel Götz</t>
+  </si>
+  <si>
+    <t>Chapter 15</t>
+  </si>
+  <si>
+    <t>Chapter 13</t>
+  </si>
+  <si>
+    <t>Chapter 16</t>
+  </si>
+  <si>
+    <t>Chapter 18</t>
+  </si>
+  <si>
+    <t>Chapter 19</t>
+  </si>
+  <si>
+    <t>Chapter 21</t>
+  </si>
+  <si>
+    <t>Chapter 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meeting of the Wardens and </t>
+  </si>
+  <si>
+    <t>Murder on the Christmasmarket and ensuing chaos</t>
+  </si>
+  <si>
+    <t>Anna catches the killer while Alexander has visions through Maximilian</t>
+  </si>
+  <si>
+    <t>The Trio gets ist name and talks about their plans to make a decision</t>
+  </si>
+  <si>
+    <t>Anna gets trained by Sabine and learns about the Wardens</t>
+  </si>
+  <si>
+    <t>Josef and August learn more about the strange happenings around the Count von Tölz and run into Count von Ingenheim</t>
+  </si>
+  <si>
+    <t>Alexander wakes up from his visions</t>
+  </si>
+  <si>
+    <t>Alexander, Helene</t>
   </si>
 </sst>
 </file>
@@ -476,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.88671875" customWidth="1"/>
@@ -663,8 +720,11 @@
       <c r="C30">
         <v>25</v>
       </c>
+      <c r="D30" t="s">
+        <v>76</v>
+      </c>
       <c r="E30" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F30" t="s">
         <v>20</v>
@@ -709,7 +769,7 @@
         <v>22</v>
       </c>
       <c r="F36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -846,10 +906,10 @@
     </row>
     <row r="49" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D49" t="s">
+        <v>57</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="F49" t="s">
         <v>50</v>
@@ -860,7 +920,7 @@
         <v>11</v>
       </c>
       <c r="D50" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>52</v>
@@ -871,24 +931,24 @@
     </row>
     <row r="51" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D51" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F51" t="s">
         <v>64</v>
-      </c>
-      <c r="F51" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="52" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D52" t="s">
+        <v>61</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E52" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="F52" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -896,19 +956,47 @@
         <v>12</v>
       </c>
       <c r="D53" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>68</v>
       </c>
       <c r="F53" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C54">
+        <v>13</v>
+      </c>
+      <c r="D54" t="s">
+        <v>78</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="55" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C55">
+        <v>16</v>
+      </c>
+      <c r="D55" t="s">
+        <v>71</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F55" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C56">
         <v>21</v>
       </c>
+      <c r="D56" t="s">
+        <v>75</v>
+      </c>
       <c r="E56" s="1" t="s">
         <v>54</v>
       </c>
@@ -918,18 +1006,79 @@
     </row>
     <row r="57" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C57">
+        <v>22</v>
+      </c>
+      <c r="D57" t="s">
+        <v>77</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="58" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C58">
+        <v>23</v>
+      </c>
+      <c r="D58" t="s">
+        <v>70</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C59">
         <v>24</v>
       </c>
-    </row>
-    <row r="58" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C58">
+      <c r="D59" t="s">
+        <v>79</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F59" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D60" t="s">
+        <v>81</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="61" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D61" t="s">
+        <v>80</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="62" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C62">
         <v>25</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="D62" t="s">
+        <v>3</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F58" t="s">
-        <v>70</v>
+      <c r="F62" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="63" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C63">
+        <v>27</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F63" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Buch und Charakter Bios
</commit_message>
<xml_diff>
--- a/docs/Buch Bayrische Nächte/Zeitlinie.xlsx
+++ b/docs/Buch Bayrische Nächte/Zeitlinie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B437D2A-10C0-4FB1-AC11-5404F361E360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301687EC-E6EF-41B7-BDEB-896471AB2670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="95">
   <si>
     <t>Year</t>
   </si>
@@ -82,28 +82,18 @@
 and only hers, capsized. Sir Charles was bheind that but no one knew. The Regatta was cancled in the following years.</t>
   </si>
   <si>
-    <t>Alexander and his brother Ludwig play on a hill. Ludwig dares himself to drive down the hill with top speed.
-Alexander cheers him up. Ludwig dies, falling of and hitting his head on a rock.</t>
-  </si>
-  <si>
     <t>June</t>
   </si>
   <si>
     <t>Friedrich, Maria sr.</t>
   </si>
   <si>
-    <t>Chapter 2</t>
-  </si>
-  <si>
     <t>Marina meets the Count Großberg to discuss the railcar project</t>
   </si>
   <si>
     <t>October</t>
   </si>
   <si>
-    <t>Chapter 3</t>
-  </si>
-  <si>
     <t>Alexander finalizes the plans for the railcar project</t>
   </si>
   <si>
@@ -119,9 +109,6 @@
     <t>December</t>
   </si>
   <si>
-    <t>Chapter 4</t>
-  </si>
-  <si>
     <t>Friedrich has an episode, that almost kills him</t>
   </si>
   <si>
@@ -134,16 +121,10 @@
     <t>Friedrich, Trautl, Elke, Maria jr.</t>
   </si>
   <si>
-    <t>Chapter 5</t>
-  </si>
-  <si>
     <t>The trio meets for the first time and ascents the mountain with the Count Großberg</t>
   </si>
   <si>
     <t>Friedrich, Marina, Alexander, Count Großberg</t>
-  </si>
-  <si>
-    <t>Chapter 6</t>
   </si>
   <si>
     <t>Marina studies the books of Großberg while the other ski. She finds out more about werewolves with Alexander. 
@@ -153,27 +134,18 @@
     <t>Friedrich, Marina, Alexander, Count Großberg, Eric</t>
   </si>
   <si>
-    <t>Chapter 7</t>
-  </si>
-  <si>
     <t>Breakfast and ski donw the slope. Friedrich hurts himself because of the other Count. A heavy storm begins. Count Großberg leaves them in the Storm and darts off.</t>
   </si>
   <si>
     <t>Friedrich, Marina, Alexander, Count Großberg, Eric, Count Ingenheim</t>
   </si>
   <si>
-    <t>Chapter 8</t>
-  </si>
-  <si>
     <t>Friedrich scouts the chalet grounds and finds the Werewolf. He hurts it badly but gets sliced himself. The others save him.</t>
   </si>
   <si>
     <t>Friedrich, Marina, Alexander, Werewolf, Eric</t>
   </si>
   <si>
-    <t>Chapter 9</t>
-  </si>
-  <si>
     <t>Marina and Alexander prepare for another Werewolf attack and have to fight against Eric. They beat him down and make themselves ready.</t>
   </si>
   <si>
@@ -183,9 +155,6 @@
     <t>Anna Siebert, Sabine, Karl</t>
   </si>
   <si>
-    <t>Chapter 1</t>
-  </si>
-  <si>
     <t>Josef Fuchsberger suspects foul play after the suspects releases</t>
   </si>
   <si>
@@ -196,12 +165,6 @@
   </si>
   <si>
     <t>Count von Ingenheim, Fuchsberger und August try to uncover the lies of the Trio but are caught in the Web of the Cult in the Karmeliterkirche next to the Christmas Market</t>
-  </si>
-  <si>
-    <t>Aelxander goes to Munich to start studying at TUM at 16 years of age</t>
-  </si>
-  <si>
-    <t>Chaper 10</t>
   </si>
   <si>
     <t>Sabine and Karl, Dianists of the Wardens, catch Anna Siebert in the villa of the Count Grossberg in Tölz</t>
@@ -211,12 +174,6 @@
 They talk about expectations of having a child.</t>
   </si>
   <si>
-    <t>Chapter 11</t>
-  </si>
-  <si>
-    <t>Chapter 12</t>
-  </si>
-  <si>
     <t>Marina arrives home with ehr huibsand Wilhelm, there she meets her son and attendance. She later has sex with her 
 husband to cope, bad dreams keeping her awake.</t>
   </si>
@@ -242,12 +199,6 @@
     <t>Friedrich, Marina, Alexander, Anna, Sabine, Helene Berthold, Nai, Sir Charles, etc.</t>
   </si>
   <si>
-    <t>Chapter 17</t>
-  </si>
-  <si>
-    <t>Chapter 14</t>
-  </si>
-  <si>
     <t>Friedrich is talking with his demented mom about life</t>
   </si>
   <si>
@@ -257,27 +208,6 @@
     <t>Marina, Wilhelm, Philipp, Christoff Bauer, Gundel Götz</t>
   </si>
   <si>
-    <t>Chapter 15</t>
-  </si>
-  <si>
-    <t>Chapter 13</t>
-  </si>
-  <si>
-    <t>Chapter 16</t>
-  </si>
-  <si>
-    <t>Chapter 18</t>
-  </si>
-  <si>
-    <t>Chapter 19</t>
-  </si>
-  <si>
-    <t>Chapter 21</t>
-  </si>
-  <si>
-    <t>Chapter 20</t>
-  </si>
-  <si>
     <t xml:space="preserve">Meeting of the Wardens and </t>
   </si>
   <si>
@@ -300,6 +230,90 @@
   </si>
   <si>
     <t>Alexander, Helene</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>Book1/13</t>
+  </si>
+  <si>
+    <t>Book1/1</t>
+  </si>
+  <si>
+    <t>Book1/2</t>
+  </si>
+  <si>
+    <t>Book1/3</t>
+  </si>
+  <si>
+    <t>Book1/4</t>
+  </si>
+  <si>
+    <t>Book1/5</t>
+  </si>
+  <si>
+    <t>Book1/6</t>
+  </si>
+  <si>
+    <t>Book1/7</t>
+  </si>
+  <si>
+    <t>Book1/8</t>
+  </si>
+  <si>
+    <t>Book1/9</t>
+  </si>
+  <si>
+    <t>Book1/10</t>
+  </si>
+  <si>
+    <t>Book1/17</t>
+  </si>
+  <si>
+    <t>Book1/11</t>
+  </si>
+  <si>
+    <t>Book1/12</t>
+  </si>
+  <si>
+    <t>Book1/18</t>
+  </si>
+  <si>
+    <t>Book1/14</t>
+  </si>
+  <si>
+    <t>Book1/15</t>
+  </si>
+  <si>
+    <t>Book1/16</t>
+  </si>
+  <si>
+    <t>Book1/19</t>
+  </si>
+  <si>
+    <t>Book1/20</t>
+  </si>
+  <si>
+    <t>Book1/21</t>
+  </si>
+  <si>
+    <t>Book1/</t>
+  </si>
+  <si>
+    <t>Alexander trying a 'science' experiment. Older schoolboys bully him for it and his brother Ludwig intervenes, sends Alexander away. He hides and hears his brother die on accident after a push, blacks it from his memories.</t>
+  </si>
+  <si>
+    <t>Alexander goes to Munich to start studying at TUM at 16 years of age</t>
+  </si>
+  <si>
+    <t>Friedrich and Maria talk again about their life together, he notices her frustration forthe first time.</t>
+  </si>
+  <si>
+    <t>Maria sr. Dies, killing herself with Friedrichs weaopn, as he walks away. He hears the shot from outside of their appartment</t>
+  </si>
+  <si>
+    <t>Alois Großbërge von Tolnzar becomes the Werewolf Fury</t>
   </si>
 </sst>
 </file>
@@ -533,12 +547,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.88671875" customWidth="1"/>
     <col min="4" max="4" width="10.44140625" customWidth="1"/>
-    <col min="5" max="5" width="105.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="109.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="70.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -562,6 +576,14 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1632</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
     <row r="4" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1850</v>
@@ -703,7 +725,7 @@
         <v>2</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>18</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -713,7 +735,7 @@
     </row>
     <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -721,364 +743,401 @@
         <v>25</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="F30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>1871</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>56</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>1882</v>
+      <c r="B34" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B35" t="s">
-        <v>14</v>
+      <c r="C35">
+        <v>6</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F35" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C36">
-        <v>10</v>
-      </c>
-      <c r="D36" t="s">
-        <v>51</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F36" t="s">
-        <v>65</v>
+      <c r="A36">
+        <v>1871</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C38">
-        <v>28</v>
-      </c>
-      <c r="D38" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F38" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C39">
-        <v>29</v>
-      </c>
-      <c r="D39" t="s">
-        <v>21</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F39" t="s">
-        <v>28</v>
+      <c r="A39">
+        <v>1882</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C41">
+        <v>10</v>
+      </c>
+      <c r="D41" t="s">
+        <v>69</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F41" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C43">
+        <v>28</v>
+      </c>
+      <c r="D43" t="s">
+        <v>70</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F43" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C44">
+        <v>29</v>
+      </c>
+      <c r="D44" t="s">
+        <v>70</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F44" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B45" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C46">
         <v>8</v>
       </c>
-      <c r="D41" t="s">
-        <v>24</v>
-      </c>
-      <c r="E41" s="1" t="s">
+      <c r="D46" t="s">
+        <v>71</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F46" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C47">
+        <v>9</v>
+      </c>
+      <c r="D47" t="s">
+        <v>71</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F47" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D48" t="s">
+        <v>72</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F48" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C42">
-        <v>9</v>
-      </c>
-      <c r="D42" t="s">
-        <v>24</v>
-      </c>
-      <c r="E42" s="1" t="s">
+    <row r="49" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D49" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F49" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D43" t="s">
-        <v>30</v>
-      </c>
-      <c r="E43" s="1" t="s">
+    <row r="50" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C50">
+        <v>10</v>
+      </c>
+      <c r="D50" t="s">
+        <v>74</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F50" t="s">
         <v>36</v>
       </c>
-      <c r="F43" t="s">
+    </row>
+    <row r="51" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D51" t="s">
+        <v>75</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D44" t="s">
-        <v>35</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F44" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C45">
-        <v>10</v>
-      </c>
-      <c r="D45" t="s">
+      <c r="F51" t="s">
         <v>38</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F45" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D46" t="s">
-        <v>41</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F46" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D47" t="s">
-        <v>44</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F47" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D48" t="s">
-        <v>47</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="49" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D49" t="s">
-        <v>57</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F49" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="50" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C50">
-        <v>11</v>
-      </c>
-      <c r="D50" t="s">
-        <v>70</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F50" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="51" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D51" t="s">
-        <v>60</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F51" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="52" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D52" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="F52" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C53">
-        <v>12</v>
-      </c>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D53" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F53" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="54" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C54">
-        <v>13</v>
-      </c>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="54" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D54" t="s">
         <v>78</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F54" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="55" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C55">
+        <v>11</v>
+      </c>
+      <c r="D55" t="s">
+        <v>79</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F55" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="56" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D56" t="s">
+        <v>80</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F56" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D57" t="s">
+        <v>81</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F57" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="58" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C58">
+        <v>12</v>
+      </c>
+      <c r="D58" t="s">
+        <v>81</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F58" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C59">
+        <v>13</v>
+      </c>
+      <c r="D59" t="s">
+        <v>82</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="60" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C60">
+        <v>16</v>
+      </c>
+      <c r="D60" t="s">
+        <v>83</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F60" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="61" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C61">
+        <v>21</v>
+      </c>
+      <c r="D61" t="s">
+        <v>84</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F61" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="62" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C62">
+        <v>22</v>
+      </c>
+      <c r="D62" t="s">
+        <v>85</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="63" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C63">
+        <v>23</v>
+      </c>
+      <c r="D63" t="s">
+        <v>79</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="64" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C64">
+        <v>24</v>
+      </c>
+      <c r="D64" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="55" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C55">
-        <v>16</v>
-      </c>
-      <c r="D55" t="s">
-        <v>71</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F55" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="56" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C56">
-        <v>21</v>
-      </c>
-      <c r="D56" t="s">
-        <v>75</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F56" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="57" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C57">
-        <v>22</v>
-      </c>
-      <c r="D57" t="s">
-        <v>77</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C58">
-        <v>23</v>
-      </c>
-      <c r="D58" t="s">
-        <v>70</v>
-      </c>
-      <c r="E58" s="1" t="s">
+      <c r="E64" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F64" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="65" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D65" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="59" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C59">
-        <v>24</v>
-      </c>
-      <c r="D59" t="s">
-        <v>79</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F59" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="60" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D60" t="s">
-        <v>81</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="61" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D61" t="s">
-        <v>80</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="62" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C62">
+      <c r="E65" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D66" t="s">
+        <v>88</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="67" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C67">
         <v>25</v>
       </c>
-      <c r="D62" t="s">
-        <v>3</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F62" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="63" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C63">
+      <c r="D67" t="s">
+        <v>89</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F67" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="68" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C68">
         <v>27</v>
       </c>
-      <c r="E63" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="D68" t="s">
         <v>89</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F68" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>